<commit_message>
feat(F-NAR-019): TREE-AUT-035 passe agent après apply
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-AUT-035.xlsx
+++ b/stories/arbres/TREE-AUT-035.xlsx
@@ -1591,17 +1591,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Nina court vers le bac, le manteau ouvert. Le sable mouillé luit, gris et froid. Une petite pelle jaune attend au bord. La pelle, je la prends ! Sa main nue serre le manche. Le bois pique, et la pelle reste collée. Je n'y arrive pas. Ton autre gant, il est où ? Nina rentre au vestiaire, les épaules basses. Les crochets sont froids sous ses doigts. Le radiateur fait tic, contre le zinc. Elle accroche le manteau, lourd, d'un coup. Le gant rouge attend contre le mur. Toi, je t'avais oublié. Pose les paumes sur le métal, un moment. Ses doigts deviennent roses, un à un. La pelle, maintenant. Nina s'agenouille près du bac. Le sable reste frais, mais ses mains tiennent.</t>
+          <t>Nina court vers le bac, le manteau ouvert. Le sable mouillé luit, gris et froid. Une petite pelle jaune attend au bord. La pelle, je la prends ! Sa main nue serre le manche. Le bois pique, et la pelle reste collée. Je n'y arrive pas. Ton autre gant, il est où ? Nina rentre au vestiaire, les épaules basses. Les crochets sont froids sous ses doigts. Le radiateur fait tic, contre le zinc. Elle accroche le manteau, lourd, d'un coup. Le gant rouge attend contre le mur. Toi, je t'avais oublié. En le ramassant, sa main nue touche le zinc. Le métal est tiède, et ses doigts s'ouvrent dessus. La pelle, maintenant. Nina s'agenouille près du bac. Le sable reste frais, mais ses mains tiennent.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Nina court vers le bac, le manteau ouvert. Le sable mouillé luit, gris et froid. Une petite pelle jaune attend au bord. La pelle, je la prends ! Sa main nue serre le manche. Le bois pique, et la pelle reste collée. Je n'y arrive pas. Ton autre gant, il est où ? Nina rentre au vestiaire, les épaules basses. Les crochets sont froids sous ses doigts. Le radiateur fait tic, contre le zinc. Elle accroche le manteau, lourd, d'un coup. Le gant rouge attend contre le mur. Toi, je t'avais oublié. Pose les paumes sur le métal, un moment. Ses doigts deviennent roses, un à un. La pelle, maintenant. Nina s'agenouille près du bac. Le sable reste frais, mais ses mains tiennent.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Nina court vers le bac, le manteau ouvert. Le sable mouillé luit, gris et froid. Une petite pelle jaune attend au bord. La pelle, je la prends ! Sa main nue serre le manche. Le bois pique, et la pelle reste collée. Je n'y arrive pas. Ton autre gant, il est où ? Nina rentre au vestiaire, les épaules basses. Les crochets sont froids sous ses doigts. Le radiateur fait tic, contre le zinc. Elle accroche le manteau, lourd, d'un coup. Le gant rouge attend contre le mur. Toi, je t'avais oublié. En le ramassant, sa main nue touche le zinc. Le métal est tiède, et ses doigts s'ouvrent dessus. La pelle, maintenant. Nina s'agenouille près du bac. Le sable reste frais, mais ses mains tiennent.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Nina court vers le bac, le manteau ouvert. Le sable mouillé luit, gris et froid. Une petite pelle jaune attend au bord. La pelle, je la prends ! Sa main nue serre le manche. Le bois pique, et la pelle reste collée. Je n'y arrive pas. Ton autre gant, il est où ? Nina rentre au vestiaire, les épaules basses. Les crochets sont froids sous ses doigts. Le radiateur fait tic, contre le zinc. Elle accroche le manteau, lourd, d'un coup. Le gant rouge attend contre le mur. Toi, je t'avais oublié. Pose les paumes sur le métal, un moment. Ses doigts deviennent roses, un à un. La pelle, maintenant. Nina s'agenouille près du bac. Le sable reste frais, mais ses mains tiennent.&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Nina court vers le bac, le manteau ouvert. Le sable mouillé luit, gris et froid. Une petite pelle jaune attend au bord. La pelle, je la prends ! Sa main nue serre le manche. Le bois pique, et la pelle reste collée. Je n'y arrive pas. Ton autre gant, il est où ? Nina rentre au vestiaire, les épaules basses. Les crochets sont froids sous ses doigts. Le radiateur fait tic, contre le zinc. Elle accroche le manteau, lourd, d'un coup. Le gant rouge attend contre le mur. Toi, je t'avais oublié. En le ramassant, sa main nue touche le zinc. Le métal est tiède, et ses doigts s'ouvrent dessus. La pelle, maintenant. Nina s'agenouille près du bac. Le sable reste frais, mais ses mains tiennent.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1753,8 +1753,8 @@
 narrateur|Elle accroche le manteau, lourd, d'un coup.
 narrateur|Le gant rouge attend contre le mur.
 enfant-f|Toi, je t'avais oublié.
-maman|Pose les paumes sur le métal, un moment.
-narrateur|Ses doigts deviennent roses, un à un.
+narrateur|En le ramassant, sa main nue touche le zinc.
+narrateur|Le métal est tiède, et ses doigts s'ouvrent dessus.
 enfant-f|La pelle, maintenant.
 narrateur|Nina s'agenouille près du bac.
 narrateur|Le sable reste frais, mais ses mains tiennent.</t>
@@ -1789,17 +1789,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Nina n'arrivait pas à tenir la pelle, près du bac. Elle a posé les mains où, pour les réchauffer ?</t>
+          <t>Nina n'arrivait pas à tenir la pelle, près du bac. Elle a posé les mains où, près du tic ?</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Nina n'arrivait pas à tenir la pelle, près du bac. Elle a posé les &lt;emphasis level="moderate"&gt;mains&lt;/emphasis&gt; où, pour les réchauffer ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Nina n'arrivait pas à tenir la pelle, près du bac. Elle a posé les &lt;emphasis level="moderate"&gt;mains&lt;/emphasis&gt; où, près du tic ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;soft&gt;&lt;slow&gt;Nina n'arrivait pas à tenir la pelle, près du bac. Elle a posé les &lt;emphasis&gt;mains&lt;/emphasis&gt; où, pour les réchauffer ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Nina n'arrivait pas à tenir la pelle, près du bac. Elle a posé les &lt;emphasis&gt;mains&lt;/emphasis&gt; où, près du tic ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -1950,7 +1950,7 @@
       <c r="AW5" t="inlineStr">
         <is>
           <t>narrateur|Nina n'arrivait pas à tenir la pelle, près du bac.
-maman|Elle a posé les mains où, pour les réchauffer ?</t>
+maman|Elle a posé les mains où, près du tic ?</t>
         </is>
       </c>
     </row>
@@ -1977,17 +1977,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Oui, sur le radiateur. Le gant rouge a retrouvé ta main. Mes doigts sont roses. Merci d'être revenue le chercher. Un grain de sable brille sur son genou. La pelle jaune attend, et cette fois elle cède.</t>
+          <t>Oui, sur le radiateur. Le gant rouge a retrouvé ta main. Mes doigts sont roses. Merci d'être revenue le chercher. Un grain de sable brille sur son genou. La pelle jaune attend, et le manche cède.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Oui, sur le radiateur. Le &lt;emphasis level="moderate"&gt;gant&lt;/emphasis&gt; rouge a retrouvé ta main. Mes doigts sont roses. Merci d'être revenue le chercher. Un grain de sable brille sur son genou. La pelle jaune attend, et cette fois elle cède.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Oui, sur le radiateur. Le &lt;emphasis level="moderate"&gt;gant&lt;/emphasis&gt; rouge a retrouvé ta main. Mes doigts sont roses. Merci d'être revenue le chercher. Un grain de sable brille sur son genou. La pelle jaune attend, et le manche cède.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Oui, sur le radiateur. Le &lt;emphasis&gt;gant&lt;/emphasis&gt; rouge a retrouvé ta main. Mes doigts sont roses. Merci d'être revenue le chercher. Un grain de sable brille sur son genou. La pelle jaune attend, et cette fois elle cède. [pause]</t>
+          <t>Oui, sur le radiateur. Le &lt;emphasis&gt;gant&lt;/emphasis&gt; rouge a retrouvé ta main. Mes doigts sont roses. Merci d'être revenue le chercher. Un grain de sable brille sur son genou. La pelle jaune attend, et le manche cède. [pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2126,7 +2126,7 @@
 enfant-f|Mes doigts sont roses.
 papa|Merci d'être revenue le chercher.
 narrateur|Un grain de sable brille sur son genou.
-narrateur|La pelle jaune attend, et cette fois elle cède.</t>
+narrateur|La pelle jaune attend, et le manche cède.</t>
         </is>
       </c>
       <c r="AX6" t="inlineStr">
@@ -3486,17 +3486,17 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Le cartable bleu attend près du vestiaire, un peu lourd. La boucle est froide sous le pouce. On ouvre ? J'ouvre. Nina ouvre la boucle, clic, sans la forcer. Un dessin à la craie est plié au fond. Elle pousse le dessin, tout au fond, sans le froisser. Le ballon sablé s'appuie contre le cartable fermé. Tu refermes ? Oui. Clic, le cartable redevient un carré fermé. Le gant rouge a retrouvé sa paire, près de la boucle.</t>
+          <t>Le cartable bleu attend près du vestiaire, un peu lourd. La boucle est froide sous le pouce. On ouvre ? J'ouvre. Nina ouvre la boucle, clic, sans la forcer. Un dessin à la craie est plié au fond. Elle pousse le dessin, tout au fond, sans le froisser. Le ballon sablé attend contre sa jambe, le temps du clic. Tu refermes ? Oui. Clic, le cartable redevient un carré fermé. Le gant rouge a retrouvé sa paire, près de la boucle.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le cartable bleu attend près du vestiaire, un peu lourd. La boucle est froide sous le pouce. On ouvre ? J'ouvre. Nina ouvre la boucle, clic, sans la forcer. Un dessin à la craie est plié au fond. Elle pousse le dessin, tout au fond, sans le froisser. Le ballon sablé s'appuie contre le cartable fermé. Tu refermes ? Oui. Clic, le cartable redevient un carré fermé. Le gant rouge a retrouvé sa paire, près de la boucle.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le cartable bleu attend près du vestiaire, un peu lourd. La boucle est froide sous le pouce. On ouvre ? J'ouvre. Nina ouvre la boucle, clic, sans la forcer. Un dessin à la craie est plié au fond. Elle pousse le dessin, tout au fond, sans le froisser. Le ballon sablé attend contre sa jambe, le temps du clic. Tu refermes ? Oui. Clic, le cartable redevient un carré fermé. Le gant rouge a retrouvé sa paire, près de la boucle.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Le cartable bleu attend près du vestiaire, un peu lourd. La boucle est froide sous le pouce. On ouvre ? J'ouvre. Nina ouvre la boucle, clic, sans la forcer. Un dessin à la craie est plié au fond. Elle pousse le dessin, tout au fond, sans le froisser. Le ballon sablé s'appuie contre le cartable fermé. Tu refermes ? Oui. Clic, le cartable redevient un carré fermé. Le gant rouge a retrouvé sa paire, près de la boucle. [pause]</t>
+          <t>Le cartable bleu attend près du vestiaire, un peu lourd. La boucle est froide sous le pouce. On ouvre ? J'ouvre. Nina ouvre la boucle, clic, sans la forcer. Un dessin à la craie est plié au fond. Elle pousse le dessin, tout au fond, sans le froisser. Le ballon sablé attend contre sa jambe, le temps du clic. Tu refermes ? Oui. Clic, le cartable redevient un carré fermé. Le gant rouge a retrouvé sa paire, près de la boucle. [pause]</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr"/>
@@ -3637,7 +3637,7 @@
 narrateur|Nina ouvre la boucle, clic, sans la forcer.
 narrateur|Un dessin à la craie est plié au fond.
 narrateur|Elle pousse le dessin, tout au fond, sans le froisser.
-narrateur|Le ballon sablé s'appuie contre le cartable fermé.
+narrateur|Le ballon sablé attend contre sa jambe, le temps du clic.
 maman|Tu refermes ?
 enfant-f|Oui.
 narrateur|Clic, le cartable redevient un carré fermé.
@@ -3860,17 +3860,17 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Le seau bleu a une anse qui brille, près du bac. Le seau ! Nina attrape l'anse trop vite. Ting, le seau bascule, vide. Il m'a échappé. Les deux gants, et plus doucement. Elle reprend l'anse, et le métal ne pique plus. Tu remplis un peu ? Oui, un peu de sable. Le sable coule, chh, dans le bleu. Nina pose le seau au bord du bac. Il est à toi, maintenant.</t>
+          <t>Le seau bleu a une anse qui brille, près du bac. Le seau ! Nina attrape l'anse trop vite. Ting, le seau bascule, vide. Il m'a échappé. Tu veux réessayer des deux mains ? Elle reprend l'anse, et le métal ne pique plus. Tu remplis un peu ? Oui, un peu de sable. Le sable coule, chh, dans le bleu. Nina pose le seau au bord du bac. Il est à toi, maintenant.</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le seau bleu a une anse qui brille, près du bac. Le seau ! Nina attrape l'anse trop vite. Ting, le seau bascule, vide. Il m'a échappé. Les deux gants, et plus doucement. Elle reprend l'anse, et le métal ne pique plus. Tu remplis un peu ? Oui, un peu de sable. Le sable coule, chh, dans le bleu. Nina pose le seau au bord du bac. Il est à toi, maintenant.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le seau bleu a une anse qui brille, près du bac. Le seau ! Nina attrape l'anse trop vite. Ting, le seau bascule, vide. Il m'a échappé. Tu veux réessayer des deux mains ? Elle reprend l'anse, et le métal ne pique plus. Tu remplis un peu ? Oui, un peu de sable. Le sable coule, chh, dans le bleu. Nina pose le seau au bord du bac. Il est à toi, maintenant.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Le seau bleu a une anse qui brille, près du bac. Le seau ! Nina attrape l'anse trop vite. Ting, le seau bascule, vide. Il m'a échappé. Les deux gants, et plus doucement. Elle reprend l'anse, et le métal ne pique plus. Tu remplis un peu ? Oui, un peu de sable. Le sable coule, chh, dans le bleu. Nina pose le seau au bord du bac. Il est à toi, maintenant. [pause]</t>
+          <t>Le seau bleu a une anse qui brille, près du bac. Le seau ! Nina attrape l'anse trop vite. Ting, le seau bascule, vide. Il m'a échappé. Tu veux réessayer des deux mains ? Elle reprend l'anse, et le métal ne pique plus. Tu remplis un peu ? Oui, un peu de sable. Le sable coule, chh, dans le bleu. Nina pose le seau au bord du bac. Il est à toi, maintenant. [pause]</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr"/>
@@ -4009,7 +4009,7 @@
 narrateur|Nina attrape l'anse trop vite.
 narrateur|Ting, le seau bascule, vide.
 enfant-f|Il m'a échappé.
-papa|Les deux gants, et plus doucement.
+papa|Tu veux réessayer des deux mains ?
 narrateur|Elle reprend l'anse, et le métal ne pique plus.
 maman|Tu remplis un peu ?
 enfant-f|Oui, un peu de sable.
@@ -4991,17 +4991,17 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Le cartable bleu attend près du vestiaire, un peu lourd. La boucle est froide sous le pouce. On ouvre ? J'ouvre. Nina ouvre la boucle, clic, sans la forcer. Un dessin à la craie est plié au fond. Elle pousse le dessin au fond, puis reprend l'anse. Le seau bleu se pose à côté de la boucle. Tu refermes ? Oui. Clic, le cartable redevient un carré fermé. Nina glisse le dessin derrière le seau, le temps d'ouvrir.</t>
+          <t>Le cartable bleu attend près du vestiaire, un peu lourd. La boucle est froide sous le pouce. On ouvre ? J'ouvre. Nina ouvre la boucle, clic, sans la forcer. Un dessin à la craie est plié au fond. Elle pousse le dessin au fond, puis reprend l'anse. Le seau bleu se pose à côté de la boucle. Tu refermes ? Oui. Clic, le cartable redevient un carré fermé. Le seau veille, et la paire rouge se touche.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le cartable bleu attend près du vestiaire, un peu lourd. La boucle est froide sous le pouce. On ouvre ? J'ouvre. Nina ouvre la boucle, clic, sans la forcer. Un dessin à la craie est plié au fond. Elle pousse le dessin au fond, puis reprend l'anse. Le seau bleu se pose à côté de la boucle. Tu refermes ? Oui. Clic, le cartable redevient un carré fermé. Nina glisse le dessin derrière le seau, le temps d'ouvrir.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le cartable bleu attend près du vestiaire, un peu lourd. La boucle est froide sous le pouce. On ouvre ? J'ouvre. Nina ouvre la boucle, clic, sans la forcer. Un dessin à la craie est plié au fond. Elle pousse le dessin au fond, puis reprend l'anse. Le seau bleu se pose à côté de la boucle. Tu refermes ? Oui. Clic, le cartable redevient un carré fermé. Le seau veille, et la paire rouge se touche.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Le cartable bleu attend près du vestiaire, un peu lourd. La boucle est froide sous le pouce. On ouvre ? J'ouvre. Nina ouvre la boucle, clic, sans la forcer. Un dessin à la craie est plié au fond. Elle pousse le dessin au fond, puis reprend l'anse. Le seau bleu se pose à côté de la boucle. Tu refermes ? Oui. Clic, le cartable redevient un carré fermé. Nina glisse le dessin derrière le seau, le temps d'ouvrir. [pause]</t>
+          <t>Le cartable bleu attend près du vestiaire, un peu lourd. La boucle est froide sous le pouce. On ouvre ? J'ouvre. Nina ouvre la boucle, clic, sans la forcer. Un dessin à la craie est plié au fond. Elle pousse le dessin au fond, puis reprend l'anse. Le seau bleu se pose à côté de la boucle. Tu refermes ? Oui. Clic, le cartable redevient un carré fermé. Le seau veille, et la paire rouge se touche. [pause]</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr"/>
@@ -5146,7 +5146,7 @@
 maman|Tu refermes ?
 enfant-f|Oui.
 narrateur|Clic, le cartable redevient un carré fermé.
-narrateur|Nina glisse le dessin derrière le seau, le temps d'ouvrir.</t>
+narrateur|Le seau veille, et la paire rouge se touche.</t>
         </is>
       </c>
       <c r="AX22" t="inlineStr">
@@ -5365,17 +5365,17 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Le doudou beige attend sur le banc, près du bac. Une oreille est pliée, un peu humide. Le doudou ! Nina le serre contre sa joue. Le tissu froid la fait grimacer. Il a froid, lui aussi. Secoue l'oreille, puis pose-le au sec. Elle secoue, et un grain de sable tombe. Elle l'assoit sur le bord de bois du bac. Il t'attend, pendant que tu creuses ? Oui, il regarde la pelle. Le tissu reprend une chaleur de main.</t>
+          <t>Le doudou beige attend sur le banc, près du bac. Une oreille est pliée, un peu humide. Le doudou ! Nina le serre contre sa joue. Le tissu froid la fait grimacer. Il a froid, lui aussi. L'oreille, tu la mets où, au sec ? Elle secoue, et un grain de sable tombe. Elle l'assoit sur le bord de bois du bac. Il t'attend, pendant que tu creuses ? Oui, il regarde la pelle. Le tissu reprend une chaleur de main.</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le doudou beige attend sur le banc, près du bac. Une oreille est pliée, un peu humide. Le doudou ! Nina le serre contre sa joue. Le tissu froid la fait grimacer. Il a froid, lui aussi. Secoue l'oreille, puis pose-le au sec. Elle secoue, et un grain de sable tombe. Elle l'assoit sur le bord de bois du bac. Il t'attend, pendant que tu creuses ? Oui, il regarde la pelle. Le tissu reprend une chaleur de main.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le doudou beige attend sur le banc, près du bac. Une oreille est pliée, un peu humide. Le doudou ! Nina le serre contre sa joue. Le tissu froid la fait grimacer. Il a froid, lui aussi. L'oreille, tu la mets où, au sec ? Elle secoue, et un grain de sable tombe. Elle l'assoit sur le bord de bois du bac. Il t'attend, pendant que tu creuses ? Oui, il regarde la pelle. Le tissu reprend une chaleur de main.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Le doudou beige attend sur le banc, près du bac. Une oreille est pliée, un peu humide. Le doudou ! Nina le serre contre sa joue. Le tissu froid la fait grimacer. Il a froid, lui aussi. Secoue l'oreille, puis pose-le au sec. Elle secoue, et un grain de sable tombe. Elle l'assoit sur le bord de bois du bac. Il t'attend, pendant que tu creuses ? Oui, il regarde la pelle. Le tissu reprend une chaleur de main. [pause]</t>
+          <t>Le doudou beige attend sur le banc, près du bac. Une oreille est pliée, un peu humide. Le doudou ! Nina le serre contre sa joue. Le tissu froid la fait grimacer. Il a froid, lui aussi. L'oreille, tu la mets où, au sec ? Elle secoue, et un grain de sable tombe. Elle l'assoit sur le bord de bois du bac. Il t'attend, pendant que tu creuses ? Oui, il regarde la pelle. Le tissu reprend une chaleur de main. [pause]</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr"/>
@@ -5515,7 +5515,7 @@
 narrateur|Nina le serre contre sa joue.
 narrateur|Le tissu froid la fait grimacer.
 enfant-f|Il a froid, lui aussi.
-maman|Secoue l'oreille, puis pose-le au sec.
+maman|L'oreille, tu la mets où, au sec ?
 narrateur|Elle secoue, et un grain de sable tombe.
 narrateur|Elle l'assoit sur le bord de bois du bac.
 papa|Il t'attend, pendant que tu creuses ?
@@ -6496,17 +6496,17 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Le cartable bleu attend près du vestiaire, un peu lourd. La boucle est froide sous le pouce. On ouvre ? J'ouvre. Nina ouvre la boucle, clic, sans la forcer. Un dessin à la craie est plié au fond. Le tissu touche la laine du manteau, au crochet. Le doudou glisse contre le cartable, l'oreille sablée. Tu refermes ? Oui. Clic, le cartable redevient un carré fermé. Nina souffle le grain, puis pousse le dessin au fond.</t>
+          <t>Le cartable bleu attend près du vestiaire, un peu lourd. La boucle est froide sous le pouce. On ouvre ? J'ouvre. Nina ouvre la boucle, clic, sans la forcer. Un dessin à la craie est plié au fond. Nina souffle le grain, puis pousse le dessin au fond. Le doudou glisse contre le cartable, l'oreille sablée. Tu refermes ? Oui. Clic, le cartable redevient un carré fermé. Le tissu touche la laine du manteau, au crochet.</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le cartable bleu attend près du vestiaire, un peu lourd. La boucle est froide sous le pouce. On ouvre ? J'ouvre. Nina ouvre la boucle, clic, sans la forcer. Un dessin à la craie est plié au fond. Le tissu touche la laine du manteau, au crochet. Le doudou glisse contre le cartable, l'oreille sablée. Tu refermes ? Oui. Clic, le cartable redevient un carré fermé. Nina souffle le grain, puis pousse le dessin au fond.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le cartable bleu attend près du vestiaire, un peu lourd. La boucle est froide sous le pouce. On ouvre ? J'ouvre. Nina ouvre la boucle, clic, sans la forcer. Un dessin à la craie est plié au fond. Nina souffle le grain, puis pousse le dessin au fond. Le doudou glisse contre le cartable, l'oreille sablée. Tu refermes ? Oui. Clic, le cartable redevient un carré fermé. Le tissu touche la laine du manteau, au crochet.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Le cartable bleu attend près du vestiaire, un peu lourd. La boucle est froide sous le pouce. On ouvre ? J'ouvre. Nina ouvre la boucle, clic, sans la forcer. Un dessin à la craie est plié au fond. Le tissu touche la laine du manteau, au crochet. Le doudou glisse contre le cartable, l'oreille sablée. Tu refermes ? Oui. Clic, le cartable redevient un carré fermé. Nina souffle le grain, puis pousse le dessin au fond. [pause]</t>
+          <t>Le cartable bleu attend près du vestiaire, un peu lourd. La boucle est froide sous le pouce. On ouvre ? J'ouvre. Nina ouvre la boucle, clic, sans la forcer. Un dessin à la craie est plié au fond. Nina souffle le grain, puis pousse le dessin au fond. Le doudou glisse contre le cartable, l'oreille sablée. Tu refermes ? Oui. Clic, le cartable redevient un carré fermé. Le tissu touche la laine du manteau, au crochet. [pause]</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr"/>
@@ -6646,12 +6646,12 @@
 enfant-f|J'ouvre.
 narrateur|Nina ouvre la boucle, clic, sans la forcer.
 narrateur|Un dessin à la craie est plié au fond.
-narrateur|Le tissu touche la laine du manteau, au crochet.
+narrateur|Nina souffle le grain, puis pousse le dessin au fond.
 narrateur|Le doudou glisse contre le cartable, l'oreille sablée.
 maman|Tu refermes ?
 enfant-f|Oui.
 narrateur|Clic, le cartable redevient un carré fermé.
-narrateur|Nina souffle le grain, puis pousse le dessin au fond.</t>
+narrateur|Le tissu touche la laine du manteau, au crochet.</t>
         </is>
       </c>
       <c r="AX30" t="inlineStr">
@@ -6870,17 +6870,17 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Nina pose un pied sur la marche du toboggan. Le plastique jaune est mouillé, glissant. Le manteau ouvert claque contre ses genoux. Je monte ! Sa main nue cherche la rampe. Le métal pince, et elle lâche tout. C'est trop froid. Le gant rouge est resté derrière. Nina revient vers le vestiaire, sans parler. Le radiateur ronronne, bas, contre le mur. Elle accroche le manteau, et les boutons tapent. L'autre gant rouge attend au pied du zinc. Tes paumes, sur le tiède. Elle pose les deux mains, et le tic marque le temps. Mes doigts reviennent. La rampe t'attendra. Nina reprend la première marche. Une goutte pend sous le rebord, ronde. Cette fois, les deux gants tiennent la rampe.</t>
+          <t>Nina pose un pied sur la marche du toboggan. Le plastique jaune est mouillé, glissant. Le manteau ouvert claque contre ses genoux. Je monte ! Sa main nue cherche la rampe. Le métal pince, et elle lâche tout. C'est trop froid. Le gant rouge est resté derrière. Nina revient vers le vestiaire, sans parler. Le radiateur ronronne, bas, contre le mur. Elle accroche le manteau, et les boutons tapent. L'autre gant rouge attend au pied du zinc. Tu as trouvé le tiède ? Elle pose les deux mains, et le tic marque le temps. Mes doigts reviennent. La rampe t'attendra. Nina reprend la première marche. Une goutte pend sous le rebord, ronde. Les deux gants tiennent la rampe, sans lâcher.</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Nina pose un pied sur la marche du toboggan. Le plastique jaune est mouillé, glissant. Le manteau ouvert claque contre ses genoux. Je monte ! Sa main nue cherche la rampe. Le métal pince, et elle lâche tout. C'est trop froid. Le gant rouge est resté derrière. Nina revient vers le vestiaire, sans parler. Le radiateur ronronne, bas, contre le mur. Elle accroche le manteau, et les boutons tapent. L'autre gant rouge attend au pied du zinc. Tes paumes, sur le tiède. Elle pose les deux mains, et le tic marque le temps. Mes doigts reviennent. La rampe t'attendra. Nina reprend la première marche. Une goutte pend sous le rebord, ronde. Cette fois, les deux gants tiennent la rampe.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Nina pose un pied sur la marche du toboggan. Le plastique jaune est mouillé, glissant. Le manteau ouvert claque contre ses genoux. Je monte ! Sa main nue cherche la rampe. Le métal pince, et elle lâche tout. C'est trop froid. Le gant rouge est resté derrière. Nina revient vers le vestiaire, sans parler. Le radiateur ronronne, bas, contre le mur. Elle accroche le manteau, et les boutons tapent. L'autre gant rouge attend au pied du zinc. Tu as trouvé le tiède ? Elle pose les deux mains, et le tic marque le temps. Mes doigts reviennent. La rampe t'attendra. Nina reprend la première marche. Une goutte pend sous le rebord, ronde. Les deux gants tiennent la rampe, sans lâcher.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Nina pose un pied sur la marche du toboggan. Le plastique jaune est mouillé, glissant. Le manteau ouvert claque contre ses genoux. Je monte ! Sa main nue cherche la rampe. Le métal pince, et elle lâche tout. C'est trop froid. Le gant rouge est resté derrière. Nina revient vers le vestiaire, sans parler. Le radiateur ronronne, bas, contre le mur. Elle accroche le manteau, et les boutons tapent. L'autre gant rouge attend au pied du zinc. Tes paumes, sur le tiède. Elle pose les deux mains, et le tic marque le temps. Mes doigts reviennent. La rampe t'attendra. Nina reprend la première marche. Une goutte pend sous le rebord, ronde. Cette fois, les deux gants tiennent la rampe.&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Nina pose un pied sur la marche du toboggan. Le plastique jaune est mouillé, glissant. Le manteau ouvert claque contre ses genoux. Je monte ! Sa main nue cherche la rampe. Le métal pince, et elle lâche tout. C'est trop froid. Le gant rouge est resté derrière. Nina revient vers le vestiaire, sans parler. Le radiateur ronronne, bas, contre le mur. Elle accroche le manteau, et les boutons tapent. L'autre gant rouge attend au pied du zinc. Tu as trouvé le tiède ? Elle pose les deux mains, et le tic marque le temps. Mes doigts reviennent. La rampe t'attendra. Nina reprend la première marche. Une goutte pend sous le rebord, ronde. Les deux gants tiennent la rampe, sans lâcher.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr"/>
@@ -7030,13 +7030,13 @@
 narrateur|Le radiateur ronronne, bas, contre le mur.
 narrateur|Elle accroche le manteau, et les boutons tapent.
 narrateur|L'autre gant rouge attend au pied du zinc.
-maman|Tes paumes, sur le tiède.
+maman|Tu as trouvé le tiède ?
 narrateur|Elle pose les deux mains, et le tic marque le temps.
 enfant-f|Mes doigts reviennent.
 papa|La rampe t'attendra.
 narrateur|Nina reprend la première marche.
 narrateur|Une goutte pend sous le rebord, ronde.
-narrateur|Cette fois, les deux gants tiennent la rampe.</t>
+narrateur|Les deux gants tiennent la rampe, sans lâcher.</t>
         </is>
       </c>
       <c r="AX32" t="inlineStr">
@@ -7068,17 +7068,17 @@
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Nina a lâché la rampe du toboggan, trop froide. Elle a posé les mains où, ensuite ?</t>
+          <t>Nina a lâché la rampe du toboggan, trop froide. Elle a posé les mains où, au vestiaire ?</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Nina a lâché la rampe du toboggan, trop froide. Elle a posé les &lt;emphasis level="moderate"&gt;mains&lt;/emphasis&gt; où, ensuite ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Nina a lâché la rampe du toboggan, trop froide. Elle a posé les &lt;emphasis level="moderate"&gt;mains&lt;/emphasis&gt; où, au vestiaire ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>&lt;soft&gt;&lt;slow&gt;Nina a lâché la rampe du toboggan, trop froide. Elle a posé les &lt;emphasis&gt;mains&lt;/emphasis&gt; où, ensuite ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Nina a lâché la rampe du toboggan, trop froide. Elle a posé les &lt;emphasis&gt;mains&lt;/emphasis&gt; où, au vestiaire ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -7229,7 +7229,7 @@
       <c r="AW33" t="inlineStr">
         <is>
           <t>narrateur|Nina a lâché la rampe du toboggan, trop froide.
-papa|Elle a posé les mains où, ensuite ?</t>
+papa|Elle a posé les mains où, au vestiaire ?</t>
         </is>
       </c>
     </row>
@@ -9139,17 +9139,17 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Le seau bleu attend au pied des marches jaunes. Le seau, maman. Nina soulève l'anse d'un coup. Ting, une goutte du rebord tombe dedans. Il a pris l'eau tout seul. Pose-le où tes pieds ne le pousseront pas. Elle le cale contre la première marche. Il est à sa place ? Oui, papa. L'anse ne pique plus sous le gant. Un oiseau crie une fois, très haut. On entend même le seau se taire.</t>
+          <t>Le seau bleu attend au pied des marches jaunes. Le seau, maman. Nina soulève l'anse d'un coup. Ting, une goutte du rebord tombe dedans. Il a pris l'eau tout seul. Où tes pieds ne le pousseront pas ? Elle le cale contre la première marche. Il est à sa place ? Oui, papa. L'anse ne pique plus sous le gant. Un oiseau crie une fois, très haut. On entend même le seau se taire.</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le seau bleu attend au pied des marches jaunes. Le seau, maman. Nina soulève l'anse d'un coup. Ting, une goutte du rebord tombe dedans. Il a pris l'eau tout seul. Pose-le où tes pieds ne le pousseront pas. Elle le cale contre la première marche. Il est à sa place ? Oui, papa. L'anse ne pique plus sous le gant. Un oiseau crie une fois, très haut. On entend même le seau se taire.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le seau bleu attend au pied des marches jaunes. Le seau, maman. Nina soulève l'anse d'un coup. Ting, une goutte du rebord tombe dedans. Il a pris l'eau tout seul. Où tes pieds ne le pousseront pas ? Elle le cale contre la première marche. Il est à sa place ? Oui, papa. L'anse ne pique plus sous le gant. Un oiseau crie une fois, très haut. On entend même le seau se taire.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Le seau bleu attend au pied des marches jaunes. Le seau, maman. Nina soulève l'anse d'un coup. Ting, une goutte du rebord tombe dedans. Il a pris l'eau tout seul. Pose-le où tes pieds ne le pousseront pas. Elle le cale contre la première marche. Il est à sa place ? Oui, papa. L'anse ne pique plus sous le gant. Un oiseau crie une fois, très haut. On entend même le seau se taire. [pause]</t>
+          <t>Le seau bleu attend au pied des marches jaunes. Le seau, maman. Nina soulève l'anse d'un coup. Ting, une goutte du rebord tombe dedans. Il a pris l'eau tout seul. Où tes pieds ne le pousseront pas ? Elle le cale contre la première marche. Il est à sa place ? Oui, papa. L'anse ne pique plus sous le gant. Un oiseau crie une fois, très haut. On entend même le seau se taire. [pause]</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr"/>
@@ -9288,7 +9288,7 @@
 narrateur|Nina soulève l'anse d'un coup.
 narrateur|Ting, une goutte du rebord tombe dedans.
 enfant-f|Il a pris l'eau tout seul.
-papa|Pose-le où tes pieds ne le pousseront pas.
+papa|Où tes pieds ne le pousseront pas ?
 narrateur|Elle le cale contre la première marche.
 maman|Il est à sa place ?
 enfant-f|Oui, papa.
@@ -10270,17 +10270,17 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Le cartable bleu attend près du vestiaire, un peu lourd. La boucle est froide sous le pouce. On ouvre ? J'ouvre. Nina ouvre la boucle, clic, sans la forcer. Un dessin à la craie est plié au fond. L'anse attend, et le cartable redevient carré. Le seau tapote la boucle, ting, puis se tait. Tu refermes ? Oui. Clic, le cartable redevient un carré fermé. Nina pousse le dessin au fond, à côté d'un crayon.</t>
+          <t>Le cartable bleu attend près du vestiaire, un peu lourd. La boucle est froide sous le pouce. On ouvre ? J'ouvre. Nina ouvre la boucle, clic, sans la forcer. Un dessin à la craie est plié au fond. Nina pousse le dessin au fond, à côté d'un crayon. Le seau tapote la boucle, ting, puis se tait. Tu refermes ? Oui. Clic, le cartable redevient un carré fermé. L'anse reste contre le cuir, sans coincer.</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le cartable bleu attend près du vestiaire, un peu lourd. La boucle est froide sous le pouce. On ouvre ? J'ouvre. Nina ouvre la boucle, clic, sans la forcer. Un dessin à la craie est plié au fond. L'anse attend, et le cartable redevient carré. Le seau tapote la boucle, ting, puis se tait. Tu refermes ? Oui. Clic, le cartable redevient un carré fermé. Nina pousse le dessin au fond, à côté d'un crayon.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le cartable bleu attend près du vestiaire, un peu lourd. La boucle est froide sous le pouce. On ouvre ? J'ouvre. Nina ouvre la boucle, clic, sans la forcer. Un dessin à la craie est plié au fond. Nina pousse le dessin au fond, à côté d'un crayon. Le seau tapote la boucle, ting, puis se tait. Tu refermes ? Oui. Clic, le cartable redevient un carré fermé. L'anse reste contre le cuir, sans coincer.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Le cartable bleu attend près du vestiaire, un peu lourd. La boucle est froide sous le pouce. On ouvre ? J'ouvre. Nina ouvre la boucle, clic, sans la forcer. Un dessin à la craie est plié au fond. L'anse attend, et le cartable redevient carré. Le seau tapote la boucle, ting, puis se tait. Tu refermes ? Oui. Clic, le cartable redevient un carré fermé. Nina pousse le dessin au fond, à côté d'un crayon. [pause]</t>
+          <t>Le cartable bleu attend près du vestiaire, un peu lourd. La boucle est froide sous le pouce. On ouvre ? J'ouvre. Nina ouvre la boucle, clic, sans la forcer. Un dessin à la craie est plié au fond. Nina pousse le dessin au fond, à côté d'un crayon. Le seau tapote la boucle, ting, puis se tait. Tu refermes ? Oui. Clic, le cartable redevient un carré fermé. L'anse reste contre le cuir, sans coincer. [pause]</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr"/>
@@ -10420,12 +10420,12 @@
 enfant-f|J'ouvre.
 narrateur|Nina ouvre la boucle, clic, sans la forcer.
 narrateur|Un dessin à la craie est plié au fond.
-narrateur|L'anse attend, et le cartable redevient carré.
+narrateur|Nina pousse le dessin au fond, à côté d'un crayon.
 narrateur|Le seau tapote la boucle, ting, puis se tait.
 maman|Tu refermes ?
 enfant-f|Oui.
 narrateur|Clic, le cartable redevient un carré fermé.
-narrateur|Nina pousse le dessin au fond, à côté d'un crayon.</t>
+narrateur|L'anse reste contre le cuir, sans coincer.</t>
         </is>
       </c>
       <c r="AX50" t="inlineStr">
@@ -12149,17 +12149,17 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>Nina s'assoit sur le siège des balançoires. Le bois est frais, et les chaînes font cling. Une main gantée tient, l'autre reste nue. J'y vais ! La chaîne nue pince sa paume. Elle ne peut pas pousser des deux côtés. Il me manque un gant. Il est près du radiateur, je crois. Nina quitte le siège, les épaules basses. Au vestiaire, le radiateur fait tic, tic. Elle accroche le manteau sur le crochet bas. La paire de gants se retrouve, rouge contre rouge. Les paumes sur le métal, tu sens ? Oui, les doigts se colorent, roses. Ils sont chauds. Les chaînes, si tu veux. Nina reprend le siège. Les deux mains tiennent, et les chaînes acceptent. La cour sent l'herbe mouillée, tout autour.</t>
+          <t>Nina s'assoit sur le siège des balançoires. Le bois est frais, et les chaînes font cling. Une main gantée tient, l'autre reste nue. J'y vais ! La chaîne nue pince sa paume. Elle ne peut pas pousser des deux côtés. Il me manque un gant. Il est près du radiateur, je crois. Nina quitte le siège, les épaules basses. Au vestiaire, le radiateur fait tic, tic. Elle accroche le manteau sur le crochet bas. La paire de gants se retrouve, rouge contre rouge. Le zinc est tiède, tu sens ? Oui, les doigts se colorent, roses. Ils sont chauds. Les chaînes, si tu veux. Nina reprend le siège. Les deux mains tiennent, et les chaînes acceptent. La cour sent l'herbe mouillée, tout autour.</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Nina s'assoit sur le siège des balançoires. Le bois est frais, et les chaînes font cling. Une main gantée tient, l'autre reste nue. J'y vais ! La chaîne nue pince sa paume. Elle ne peut pas pousser des deux côtés. Il me manque un gant. Il est près du radiateur, je crois. Nina quitte le siège, les épaules basses. Au vestiaire, le radiateur fait tic, tic. Elle accroche le manteau sur le crochet bas. La paire de gants se retrouve, rouge contre rouge. Les paumes sur le métal, tu sens ? Oui, les doigts se colorent, roses. Ils sont chauds. Les chaînes, si tu veux. Nina reprend le siège. Les deux mains tiennent, et les chaînes acceptent. La cour sent l'herbe mouillée, tout autour.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Nina s'assoit sur le siège des balançoires. Le bois est frais, et les chaînes font cling. Une main gantée tient, l'autre reste nue. J'y vais ! La chaîne nue pince sa paume. Elle ne peut pas pousser des deux côtés. Il me manque un gant. Il est près du radiateur, je crois. Nina quitte le siège, les épaules basses. Au vestiaire, le radiateur fait tic, tic. Elle accroche le manteau sur le crochet bas. La paire de gants se retrouve, rouge contre rouge. Le zinc est tiède, tu sens ? Oui, les doigts se colorent, roses. Ils sont chauds. Les chaînes, si tu veux. Nina reprend le siège. Les deux mains tiennent, et les chaînes acceptent. La cour sent l'herbe mouillée, tout autour.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Nina s'assoit sur le siège des balançoires. Le bois est frais, et les chaînes font cling. Une main gantée tient, l'autre reste nue. J'y vais ! La chaîne nue pince sa paume. Elle ne peut pas pousser des deux côtés. Il me manque un gant. Il est près du radiateur, je crois. Nina quitte le siège, les épaules basses. Au vestiaire, le radiateur fait tic, tic. Elle accroche le manteau sur le crochet bas. La paire de gants se retrouve, rouge contre rouge. Les paumes sur le métal, tu sens ? Oui, les doigts se colorent, roses. Ils sont chauds. Les chaînes, si tu veux. Nina reprend le siège. Les deux mains tiennent, et les chaînes acceptent. La cour sent l'herbe mouillée, tout autour.&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Nina s'assoit sur le siège des balançoires. Le bois est frais, et les chaînes font cling. Une main gantée tient, l'autre reste nue. J'y vais ! La chaîne nue pince sa paume. Elle ne peut pas pousser des deux côtés. Il me manque un gant. Il est près du radiateur, je crois. Nina quitte le siège, les épaules basses. Au vestiaire, le radiateur fait tic, tic. Elle accroche le manteau sur le crochet bas. La paire de gants se retrouve, rouge contre rouge. Le zinc est tiède, tu sens ? Oui, les doigts se colorent, roses. Ils sont chauds. Les chaînes, si tu veux. Nina reprend le siège. Les deux mains tiennent, et les chaînes acceptent. La cour sent l'herbe mouillée, tout autour.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr"/>
@@ -12309,7 +12309,7 @@
 narrateur|Au vestiaire, le radiateur fait tic, tic.
 narrateur|Elle accroche le manteau sur le crochet bas.
 narrateur|La paire de gants se retrouve, rouge contre rouge.
-papa|Les paumes sur le métal, tu sens ?
+papa|Le zinc est tiède, tu sens ?
 narrateur|Oui, les doigts se colorent, roses.
 enfant-f|Ils sont chauds.
 maman|Les chaînes, si tu veux.
@@ -12535,17 +12535,17 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>Oui, les mains sur le radiateur. La paire de gants est complète. Je peux tenir les deux chaînes. Merci d'avoir écouté le tic. Une ombre d'oiseau passe sur le bois. Le siège reste frais, mais les paumes tiennent.</t>
+          <t>Oui, les mains sur le radiateur. La paire de gants est complète. Je peux tenir les deux chaînes. Merci, tes deux mains tiennent. Une ombre d'oiseau passe sur le bois. Le siège reste frais, mais les paumes tiennent.</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Oui, les mains sur le radiateur. La paire de &lt;emphasis level="moderate"&gt;gant&lt;/emphasis&gt;s est complète. Je peux tenir les deux chaînes. Merci d'avoir écouté le tic. Une ombre d'oiseau passe sur le bois. Le siège reste frais, mais les paumes tiennent.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Oui, les mains sur le radiateur. La paire de &lt;emphasis level="moderate"&gt;gant&lt;/emphasis&gt;s est complète. Je peux tenir les deux chaînes. Merci, tes deux mains tiennent. Une ombre d'oiseau passe sur le bois. Le siège reste frais, mais les paumes tiennent.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>Oui, les mains sur le radiateur. La paire de &lt;emphasis&gt;gant&lt;/emphasis&gt;s est complète. Je peux tenir les deux chaînes. Merci d'avoir écouté le tic. Une ombre d'oiseau passe sur le bois. Le siège reste frais, mais les paumes tiennent. [pause]</t>
+          <t>Oui, les mains sur le radiateur. La paire de &lt;emphasis&gt;gant&lt;/emphasis&gt;s est complète. Je peux tenir les deux chaînes. Merci, tes deux mains tiennent. Une ombre d'oiseau passe sur le bois. Le siège reste frais, mais les paumes tiennent. [pause]</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr"/>
@@ -12682,7 +12682,7 @@
           <t>papa|Oui, les mains sur le radiateur.
 maman|La paire de gants est complète.
 enfant-f|Je peux tenir les deux chaînes.
-papa|Merci d'avoir écouté le tic.
+papa|Merci, tes deux mains tiennent.
 narrateur|Une ombre d'oiseau passe sur le bois.
 narrateur|Le siège reste frais, mais les paumes tiennent.</t>
         </is>
@@ -13485,17 +13485,17 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>Le ballon dort entre les pieds du pilier, loin des chaînes. Il ne s'envole plus. Tu l'as mis trop haut, d'abord. Nina croque la pomme, les deux gants fermés sur le fruit. Le fil d'argent coupe le ciel de la vitre, très net. Les chaînes se taisent, de l'autre côté. Moi, je tiens les deux, maintenant. Le radiateur tic, et le bois du préau sent le sec.</t>
+          <t>Le ballon dort entre les pieds du pilier, loin des chaînes. Il ne s'envole plus. Tu l'as mis trop haut, au premier essai. Nina croque la pomme, les deux gants fermés sur le fruit. Le fil d'argent coupe le ciel de la vitre, très net. Les chaînes se taisent, de l'autre côté. Moi, je tiens les deux, maintenant. Le radiateur tic, et le bois du préau sent le sec.</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le ballon dort entre les pieds du pilier, loin des chaînes. Il ne s'envole plus. Tu l'as mis trop haut, d'abord. Nina croque la pomme, les deux gants fermés sur le fruit. Le &lt;emphasis level="moderate"&gt;fil d'argent&lt;/emphasis&gt; coupe le ciel de la vitre, très net. Les chaînes se taisent, de l'autre côté. Moi, je tiens les deux, maintenant. Le radiateur tic, et le bois du préau sent le sec.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le ballon dort entre les pieds du pilier, loin des chaînes. Il ne s'envole plus. Tu l'as mis trop haut, au premier essai. Nina croque la pomme, les deux gants fermés sur le fruit. Le &lt;emphasis level="moderate"&gt;fil d'argent&lt;/emphasis&gt; coupe le ciel de la vitre, très net. Les chaînes se taisent, de l'autre côté. Moi, je tiens les deux, maintenant. Le radiateur tic, et le bois du préau sent le sec.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le ballon dort entre les pieds du pilier, loin des chaînes. Il ne s'envole plus. Tu l'as mis trop haut, d'abord. Nina croque la pomme, les deux gants fermés sur le fruit. Le &lt;emphasis&gt;fil d'argent&lt;/emphasis&gt; coupe le ciel de la vitre, très net. Les chaînes se taisent, de l'autre côté. Moi, je tiens les deux, maintenant. Le radiateur tic, et le bois du préau sent le sec.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le ballon dort entre les pieds du pilier, loin des chaînes. Il ne s'envole plus. Tu l'as mis trop haut, au premier essai. Nina croque la pomme, les deux gants fermés sur le fruit. Le &lt;emphasis&gt;fil d'argent&lt;/emphasis&gt; coupe le ciel de la vitre, très net. Les chaînes se taisent, de l'autre côté. Moi, je tiens les deux, maintenant. Le radiateur tic, et le bois du préau sent le sec.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr"/>
@@ -13635,7 +13635,7 @@
         <is>
           <t>narrateur|Le ballon dort entre les pieds du pilier, loin des chaînes.
 enfant-f|Il ne s'envole plus.
-maman|Tu l'as mis trop haut, d'abord.
+maman|Tu l'as mis trop haut, au premier essai.
 narrateur|Nina croque la pomme, les deux gants fermés sur le fruit.
 narrateur|Le fil d'argent coupe le ciel de la vitre, très net.
 papa|Les chaînes se taisent, de l'autre côté.
@@ -15550,17 +15550,17 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Le cartable bleu attend près du vestiaire, un peu lourd. La boucle est froide sous le pouce. On ouvre ? J'ouvre. Nina ouvre la boucle, clic, sans la forcer. Un dessin à la craie est plié au fond. Ting, le cartable et le seau se taisent ensemble. Le seau bleu reste à côté de la boucle fermée. Tu refermes ? Oui. Clic, le cartable redevient un carré fermé. Nina pousse le dessin au fond, puis tapote l'anse.</t>
+          <t>Le cartable bleu attend près du vestiaire, un peu lourd. La boucle est froide sous le pouce. On ouvre ? J'ouvre. Nina ouvre la boucle, clic, sans la forcer. Un dessin à la craie est plié au fond. Nina pousse le dessin au fond, puis tapote l'anse. Le seau bleu reste à côté de la boucle. Tu refermes ? Oui. Clic, le cartable redevient un carré fermé. Ting, le cartable et le seau se taisent ensemble.</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le cartable bleu attend près du vestiaire, un peu lourd. La boucle est froide sous le pouce. On ouvre ? J'ouvre. Nina ouvre la boucle, clic, sans la forcer. Un dessin à la craie est plié au fond. Ting, le cartable et le seau se taisent ensemble. Le seau bleu reste à côté de la boucle fermée. Tu refermes ? Oui. Clic, le cartable redevient un carré fermé. Nina pousse le dessin au fond, puis tapote l'anse.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le cartable bleu attend près du vestiaire, un peu lourd. La boucle est froide sous le pouce. On ouvre ? J'ouvre. Nina ouvre la boucle, clic, sans la forcer. Un dessin à la craie est plié au fond. Nina pousse le dessin au fond, puis tapote l'anse. Le seau bleu reste à côté de la boucle. Tu refermes ? Oui. Clic, le cartable redevient un carré fermé. Ting, le cartable et le seau se taisent ensemble.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>Le cartable bleu attend près du vestiaire, un peu lourd. La boucle est froide sous le pouce. On ouvre ? J'ouvre. Nina ouvre la boucle, clic, sans la forcer. Un dessin à la craie est plié au fond. Ting, le cartable et le seau se taisent ensemble. Le seau bleu reste à côté de la boucle fermée. Tu refermes ? Oui. Clic, le cartable redevient un carré fermé. Nina pousse le dessin au fond, puis tapote l'anse. [pause]</t>
+          <t>Le cartable bleu attend près du vestiaire, un peu lourd. La boucle est froide sous le pouce. On ouvre ? J'ouvre. Nina ouvre la boucle, clic, sans la forcer. Un dessin à la craie est plié au fond. Nina pousse le dessin au fond, puis tapote l'anse. Le seau bleu reste à côté de la boucle. Tu refermes ? Oui. Clic, le cartable redevient un carré fermé. Ting, le cartable et le seau se taisent ensemble. [pause]</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr"/>
@@ -15700,12 +15700,12 @@
 enfant-f|J'ouvre.
 narrateur|Nina ouvre la boucle, clic, sans la forcer.
 narrateur|Un dessin à la craie est plié au fond.
-narrateur|Ting, le cartable et le seau se taisent ensemble.
-narrateur|Le seau bleu reste à côté de la boucle fermée.
+narrateur|Nina pousse le dessin au fond, puis tapote l'anse.
+narrateur|Le seau bleu reste à côté de la boucle.
 maman|Tu refermes ?
 enfant-f|Oui.
 narrateur|Clic, le cartable redevient un carré fermé.
-narrateur|Nina pousse le dessin au fond, puis tapote l'anse.</t>
+narrateur|Ting, le cartable et le seau se taisent ensemble.</t>
         </is>
       </c>
       <c r="AX78" t="inlineStr">
@@ -17423,7 +17423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -17536,6 +17536,13 @@
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>